<commit_message>
update: sync latest chat records to markdown
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/test_result/result.xlsx
+++ b/test_result/result.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="115">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="130">
   <si>
     <t>问题</t>
   </si>
@@ -192,6 +192,51 @@
   </si>
   <si>
     <t>[商机表]商机编号为“O20241202”的预计毛利（est_gross_profit）是多少？</t>
+  </si>
+  <si>
+    <t>[项目表] 所有项目的“营业收入”总和是多少？</t>
+  </si>
+  <si>
+    <t>[商机表] 在所有“生命状态”为“活跃”的商机中，哪一个“所属业务单元”拥有的活跃商机数量最多？</t>
+  </si>
+  <si>
+    <t>央国企</t>
+  </si>
+  <si>
+    <t>[合同表] 最终用户为“中国建设银行股份有限公司”的所有合同，其平均毛利率是多少？</t>
+  </si>
+  <si>
+    <t>[项目表] 在项目表中，有多少个项目的“已确认比例”达到或超过了 100%（即 1.0）？</t>
+  </si>
+  <si>
+    <t>[商机表] 客户名称为“腾讯科技（深圳）有限公司”的商机中，一共出现了哪几种不同的“不纳入原因”？</t>
+  </si>
+  <si>
+    <t>合同风险过高, 商务条款无法达成一致, 项目延期, 技术方案需重新评估, 客户内部调整, 竞争对手优势明显, 客户预算不足</t>
+  </si>
+  <si>
+    <t>[合同表] 按合同名称汇总，哪一个合同贡献的“净利润(元)”总和最高？</t>
+  </si>
+  <si>
+    <t>中国工商银行股份有限公司数据治理合同</t>
+  </si>
+  <si>
+    <t>[项目表] 在所有项目中，“合同毛利”金额最高的是哪一个项目？</t>
+  </si>
+  <si>
+    <t>招商银行股份有限公司业务中台交付项目</t>
+  </si>
+  <si>
+    <t>[合同表] 在所有的合同记录中，一共涉及了多少位不同的销售“负责人”？</t>
+  </si>
+  <si>
+    <t>[项目表] 统计项目表中，存在多少个“收入毛利”小于 0 的亏损项目？</t>
+  </si>
+  <si>
+    <t>[项目表] 所有交付项目中，“项目开始时间”最早的是哪一个项目？对应的启动日期是哪一天？</t>
+  </si>
+  <si>
+    <t>京东集团股份有限公司数据治理交付项目，2025-02-18</t>
   </si>
   <si>
     <t>[商机表] 商机被排除/流失的主要原因有哪些？这揭示了业务推进中的什么核心短板？请给出针对 Top3 原因的改进建议。</t>
@@ -1324,7 +1369,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1339,6 +1384,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -1883,7 +1931,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:C71"/>
+  <dimension ref="A1:C81"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="13.5" outlineLevelCol="2"/>
   <cols>
     <col min="1" max="1" width="106.875" customWidth="1"/>
@@ -2221,244 +2269,324 @@
         <v>83</v>
       </c>
     </row>
-    <row r="42" ht="324" spans="1:2">
-      <c r="A42" t="s">
+    <row r="42" spans="1:2">
+      <c r="A42" s="4" t="s">
         <v>55</v>
       </c>
-      <c r="B42" s="4" t="s">
+      <c r="B42" s="5">
+        <v>2302277347.66</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="43" ht="189" spans="1:2">
-      <c r="A43" t="s">
+      <c r="B43" s="6" t="s">
         <v>57</v>
       </c>
-      <c r="B43" s="4" t="s">
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" t="s">
         <v>58</v>
       </c>
-    </row>
-    <row r="44" ht="256.5" spans="1:2">
-      <c r="A44" t="s">
+      <c r="B44" s="5">
+        <v>0.328675</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" t="s">
         <v>59</v>
       </c>
-      <c r="B44" s="4" t="s">
+      <c r="B45" s="5">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="46" ht="27" spans="1:2">
+      <c r="A46" t="s">
         <v>60</v>
       </c>
-    </row>
-    <row r="45" ht="391.5" spans="1:2">
-      <c r="A45" t="s">
+      <c r="B46" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="B45" s="4" t="s">
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" t="s">
         <v>62</v>
       </c>
-    </row>
-    <row r="46" ht="270" spans="1:2">
-      <c r="A46" t="s">
+      <c r="B47" s="6" t="s">
         <v>63</v>
       </c>
-      <c r="B46" s="4" t="s">
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="47" ht="256.5" spans="1:2">
-      <c r="A47" t="s">
+      <c r="B48" s="6" t="s">
         <v>65</v>
       </c>
-      <c r="B47" s="4" t="s">
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" t="s">
         <v>66</v>
       </c>
-    </row>
-    <row r="48" ht="175.5" spans="1:2">
-      <c r="A48" t="s">
+      <c r="B49" s="5">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
         <v>67</v>
       </c>
-      <c r="B48" s="4" t="s">
+      <c r="B50" s="5">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" t="s">
         <v>68</v>
       </c>
-    </row>
-    <row r="49" ht="229.5" spans="1:2">
-      <c r="A49" t="s">
+      <c r="B51" s="6" t="s">
         <v>69</v>
       </c>
-      <c r="B49" s="4" t="s">
+    </row>
+    <row r="52" ht="324" spans="1:2">
+      <c r="A52" t="s">
         <v>70</v>
       </c>
-    </row>
-    <row r="50" ht="270" spans="1:2">
-      <c r="A50" t="s">
+      <c r="B52" s="6" t="s">
         <v>71</v>
       </c>
-      <c r="B50" s="4" t="s">
+    </row>
+    <row r="53" ht="189" spans="1:2">
+      <c r="A53" t="s">
         <v>72</v>
       </c>
-    </row>
-    <row r="51" ht="256.5" spans="1:2">
-      <c r="A51" s="4" t="s">
+      <c r="B53" s="6" t="s">
         <v>73</v>
-      </c>
-      <c r="B51" s="4" t="s">
-        <v>74</v>
-      </c>
-    </row>
-    <row r="52" ht="283.5" spans="1:2">
-      <c r="A52" t="s">
-        <v>75</v>
-      </c>
-      <c r="B52" s="4" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="53" ht="310.5" spans="1:2">
-      <c r="A53" t="s">
-        <v>77</v>
-      </c>
-      <c r="B53" s="4" t="s">
-        <v>78</v>
       </c>
     </row>
     <row r="54" ht="256.5" spans="1:2">
       <c r="A54" t="s">
+        <v>74</v>
+      </c>
+      <c r="B54" s="6" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="55" ht="391.5" spans="1:2">
+      <c r="A55" t="s">
+        <v>76</v>
+      </c>
+      <c r="B55" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="56" ht="270" spans="1:2">
+      <c r="A56" t="s">
+        <v>78</v>
+      </c>
+      <c r="B56" s="6" t="s">
         <v>79</v>
       </c>
-      <c r="B54" s="4" t="s">
+    </row>
+    <row r="57" ht="256.5" spans="1:2">
+      <c r="A57" t="s">
         <v>80</v>
       </c>
-    </row>
-    <row r="55" ht="297" spans="1:2">
-      <c r="A55" t="s">
+      <c r="B57" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="B55" s="4" t="s">
+    </row>
+    <row r="58" ht="175.5" spans="1:2">
+      <c r="A58" t="s">
         <v>82</v>
       </c>
-    </row>
-    <row r="56" ht="351" spans="1:2">
-      <c r="A56" t="s">
+      <c r="B58" s="6" t="s">
         <v>83</v>
       </c>
-      <c r="B56" s="4" t="s">
+    </row>
+    <row r="59" ht="229.5" spans="1:2">
+      <c r="A59" t="s">
         <v>84</v>
       </c>
-    </row>
-    <row r="57" ht="189" spans="1:2">
-      <c r="A57" t="s">
+      <c r="B59" s="6" t="s">
         <v>85</v>
       </c>
-      <c r="B57" s="4" t="s">
+    </row>
+    <row r="60" ht="270" spans="1:2">
+      <c r="A60" t="s">
         <v>86</v>
       </c>
-    </row>
-    <row r="58" ht="256.5" spans="1:2">
-      <c r="A58" t="s">
+      <c r="B60" s="6" t="s">
         <v>87</v>
       </c>
-      <c r="B58" s="5" t="s">
+    </row>
+    <row r="61" ht="256.5" spans="1:2">
+      <c r="A61" s="6" t="s">
         <v>88</v>
       </c>
-    </row>
-    <row r="59" ht="202.5" spans="1:2">
-      <c r="A59" t="s">
+      <c r="B61" s="6" t="s">
         <v>89</v>
       </c>
-      <c r="B59" s="5" t="s">
+    </row>
+    <row r="62" ht="283.5" spans="1:2">
+      <c r="A62" t="s">
         <v>90</v>
       </c>
-    </row>
-    <row r="60" ht="405" spans="1:2">
-      <c r="A60" t="s">
+      <c r="B62" s="6" t="s">
         <v>91</v>
       </c>
-      <c r="B60" s="5" t="s">
+    </row>
+    <row r="63" ht="310.5" spans="1:2">
+      <c r="A63" t="s">
         <v>92</v>
       </c>
-    </row>
-    <row r="61" ht="337.5" spans="1:2">
-      <c r="A61" t="s">
+      <c r="B63" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="B61" s="5" t="s">
+    </row>
+    <row r="64" ht="256.5" spans="1:2">
+      <c r="A64" t="s">
         <v>94</v>
       </c>
-    </row>
-    <row r="62" ht="175.5" spans="1:2">
-      <c r="A62" t="s">
+      <c r="B64" s="6" t="s">
         <v>95</v>
       </c>
-      <c r="B62" s="5" t="s">
+    </row>
+    <row r="65" ht="297" spans="1:2">
+      <c r="A65" t="s">
         <v>96</v>
       </c>
-    </row>
-    <row r="63" ht="216" spans="1:2">
-      <c r="A63" t="s">
+      <c r="B65" s="6" t="s">
         <v>97</v>
       </c>
-      <c r="B63" s="5" t="s">
+    </row>
+    <row r="66" ht="351" spans="1:2">
+      <c r="A66" t="s">
         <v>98</v>
       </c>
-    </row>
-    <row r="64" ht="216" spans="1:2">
-      <c r="A64" t="s">
+      <c r="B66" s="6" t="s">
         <v>99</v>
       </c>
-      <c r="B64" s="5" t="s">
+    </row>
+    <row r="67" ht="189" spans="1:2">
+      <c r="A67" t="s">
         <v>100</v>
       </c>
-    </row>
-    <row r="65" ht="189" spans="1:2">
-      <c r="A65" t="s">
+      <c r="B67" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="B65" s="5" t="s">
+    </row>
+    <row r="68" ht="256.5" spans="1:2">
+      <c r="A68" t="s">
         <v>102</v>
       </c>
-    </row>
-    <row r="66" ht="189" spans="1:2">
-      <c r="A66" t="s">
+      <c r="B68" s="6" t="s">
         <v>103</v>
-      </c>
-      <c r="B66" s="5" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="67" ht="202.5" spans="1:2">
-      <c r="A67" t="s">
-        <v>105</v>
-      </c>
-      <c r="B67" s="5" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="68" ht="189" spans="1:2">
-      <c r="A68" t="s">
-        <v>107</v>
-      </c>
-      <c r="B68" s="5" t="s">
-        <v>108</v>
       </c>
     </row>
     <row r="69" ht="202.5" spans="1:2">
       <c r="A69" t="s">
+        <v>104</v>
+      </c>
+      <c r="B69" s="6" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="70" ht="405" spans="1:2">
+      <c r="A70" t="s">
+        <v>106</v>
+      </c>
+      <c r="B70" s="6" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="71" ht="337.5" spans="1:2">
+      <c r="A71" t="s">
+        <v>108</v>
+      </c>
+      <c r="B71" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="B69" s="5" t="s">
+    </row>
+    <row r="72" ht="175.5" spans="1:2">
+      <c r="A72" t="s">
         <v>110</v>
       </c>
-    </row>
-    <row r="70" ht="216" spans="1:2">
-      <c r="A70" t="s">
+      <c r="B72" s="6" t="s">
         <v>111</v>
       </c>
-      <c r="B70" s="5" t="s">
+    </row>
+    <row r="73" ht="216" spans="1:2">
+      <c r="A73" t="s">
         <v>112</v>
       </c>
-    </row>
-    <row r="71" ht="175.5" spans="1:2">
-      <c r="A71" t="s">
+      <c r="B73" s="6" t="s">
         <v>113</v>
       </c>
-      <c r="B71" s="5" t="s">
+    </row>
+    <row r="74" ht="216" spans="1:2">
+      <c r="A74" t="s">
         <v>114</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="75" ht="189" spans="1:2">
+      <c r="A75" t="s">
+        <v>116</v>
+      </c>
+      <c r="B75" s="6" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="76" ht="189" spans="1:2">
+      <c r="A76" t="s">
+        <v>118</v>
+      </c>
+      <c r="B76" s="6" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="77" ht="202.5" spans="1:2">
+      <c r="A77" t="s">
+        <v>120</v>
+      </c>
+      <c r="B77" s="6" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="78" ht="189" spans="1:2">
+      <c r="A78" t="s">
+        <v>122</v>
+      </c>
+      <c r="B78" s="6" t="s">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="79" ht="202.5" spans="1:2">
+      <c r="A79" t="s">
+        <v>124</v>
+      </c>
+      <c r="B79" s="6" t="s">
+        <v>125</v>
+      </c>
+    </row>
+    <row r="80" ht="216" spans="1:2">
+      <c r="A80" t="s">
+        <v>126</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="81" ht="175.5" spans="1:2">
+      <c r="A81" t="s">
+        <v>128</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>129</v>
       </c>
     </row>
   </sheetData>

</xml_diff>